<commit_message>
Verify workbook styling and dim suppressed rows
</commit_message>
<xml_diff>
--- a/fixtures/FTC_Competition_Robot_BOM_2026-10-23.xlsx
+++ b/fixtures/FTC_Competition_Robot_BOM_2026-10-23.xlsx
@@ -950,20 +950,20 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="0" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">Spare Gear</t>
         </is>
       </c>
-      <c r="B2" s="0">
+      <c r="B2" s="23">
         <v>4</v>
       </c>
-      <c r="C2" s="0" t="inlineStr">
+      <c r="C2" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">FTC Competition Robot &gt; Spare Gear &lt;1&gt;; FTC Competition Robot &gt; Spare Gear &lt;2&gt;; FTC Competition Robot &gt; Spare Gear &lt;3&gt;; FTC Competition Robot &gt; Spare Gear &lt;4&gt;</t>
         </is>
       </c>
-      <c r="D2" s="17" t="inlineStr">
+      <c r="D2" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">https://cad.onshape.com/documents/robot/w/fixture/e/gears</t>
         </is>

</xml_diff>